<commit_message>
#14 Parts Names Updated.
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/eSpark_BOM.xlsx
+++ b/Deliverables/BOM/eSpark_BOM.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="773" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="773" uniqueCount="256">
   <si>
     <t>Component list</t>
   </si>
@@ -734,9 +734,6 @@
     <t>C12018</t>
   </si>
   <si>
-    <t>Peripheral</t>
-  </si>
-  <si>
     <t>WJ2EDGK-5.08-3P</t>
   </si>
   <si>
@@ -786,6 +783,12 @@
   </si>
   <si>
     <t xml:space="preserve">  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMA Cable </t>
+  </si>
+  <si>
+    <t>Antenna</t>
   </si>
 </sst>
 </file>
@@ -1499,6 +1502,98 @@
     <xf numFmtId="0" fontId="19" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="15" fillId="3" borderId="22" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="5" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="5" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="2" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="24" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="2" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1511,10 +1606,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1522,6 +1617,14 @@
     </xf>
     <xf numFmtId="0" fontId="17" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1531,110 +1634,10 @@
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="3" borderId="22" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="5" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="6" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="5" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="2" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="24" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="2" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2067,15 +2070,15 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="77"/>
-      <c r="L1" s="77"/>
-      <c r="M1" s="77"/>
-      <c r="N1" s="77"/>
-      <c r="O1" s="77"/>
-      <c r="P1" s="77"/>
-      <c r="Q1" s="77"/>
-      <c r="R1" s="77"/>
-      <c r="S1" s="78"/>
+      <c r="K1" s="107"/>
+      <c r="L1" s="107"/>
+      <c r="M1" s="107"/>
+      <c r="N1" s="107"/>
+      <c r="O1" s="107"/>
+      <c r="P1" s="107"/>
+      <c r="Q1" s="107"/>
+      <c r="R1" s="107"/>
+      <c r="S1" s="108"/>
     </row>
     <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2086,7 +2089,7 @@
       </c>
       <c r="E2" s="11"/>
       <c r="F2" s="53" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="G2" s="12"/>
       <c r="H2" s="4"/>
@@ -2125,7 +2128,7 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="5"/>
-      <c r="S3" s="79"/>
+      <c r="S3" s="109"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -2150,7 +2153,7 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
-      <c r="S4" s="80"/>
+      <c r="S4" s="110"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -2175,7 +2178,7 @@
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
       <c r="R5" s="6"/>
-      <c r="S5" s="80"/>
+      <c r="S5" s="110"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -2196,7 +2199,7 @@
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
-      <c r="S6" s="80"/>
+      <c r="S6" s="110"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -2217,7 +2220,7 @@
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
-      <c r="S7" s="80"/>
+      <c r="S7" s="110"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -2238,7 +2241,7 @@
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
-      <c r="S8" s="80"/>
+      <c r="S8" s="110"/>
     </row>
     <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -2299,7 +2302,7 @@
     </row>
     <row r="10" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
-      <c r="B10" s="94">
+      <c r="B10" s="84">
         <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
@@ -2340,78 +2343,78 @@
       <c r="N10" s="45">
         <v>40</v>
       </c>
-      <c r="O10" s="110" t="s">
+      <c r="O10" s="96" t="s">
         <v>193</v>
       </c>
       <c r="P10" s="50">
         <v>2.3900000000000001E-2</v>
       </c>
-      <c r="Q10" s="114">
+      <c r="Q10" s="100">
         <f>P10*N10</f>
         <v>0.95600000000000007</v>
       </c>
       <c r="R10" s="45"/>
-      <c r="S10" s="87"/>
+      <c r="S10" s="77"/>
     </row>
     <row r="11" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
-      <c r="B11" s="94">
+      <c r="B11" s="84">
         <f t="shared" ref="B11:B46" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
-      <c r="C11" s="88" t="s">
+      <c r="C11" s="78" t="s">
         <v>7</v>
       </c>
-      <c r="D11" s="89" t="s">
+      <c r="D11" s="79" t="s">
         <v>21</v>
       </c>
-      <c r="E11" s="91" t="s">
+      <c r="E11" s="81" t="s">
         <v>53</v>
       </c>
-      <c r="F11" s="91" t="s">
+      <c r="F11" s="81" t="s">
         <v>81</v>
       </c>
-      <c r="G11" s="109" t="s">
+      <c r="G11" s="95" t="s">
         <v>101</v>
       </c>
-      <c r="H11" s="90" t="s">
+      <c r="H11" s="80" t="s">
         <v>125</v>
       </c>
-      <c r="I11" s="91" t="s">
+      <c r="I11" s="81" t="s">
         <v>226</v>
       </c>
-      <c r="J11" s="91" t="s">
+      <c r="J11" s="81" t="s">
         <v>227</v>
       </c>
-      <c r="K11" s="90" t="s">
+      <c r="K11" s="80" t="s">
         <v>162</v>
       </c>
-      <c r="L11" s="91">
+      <c r="L11" s="81">
         <v>3</v>
       </c>
-      <c r="M11" s="90">
+      <c r="M11" s="80">
         <f t="shared" ref="M11:M46" si="1">L11*10</f>
         <v>30</v>
       </c>
-      <c r="N11" s="91">
+      <c r="N11" s="81">
         <v>100</v>
       </c>
-      <c r="O11" s="111" t="s">
+      <c r="O11" s="97" t="s">
         <v>193</v>
       </c>
-      <c r="P11" s="92">
+      <c r="P11" s="82">
         <v>3.0000000000000001E-3</v>
       </c>
-      <c r="Q11" s="115">
+      <c r="Q11" s="101">
         <f t="shared" ref="Q11:Q46" si="2">P11*N11</f>
         <v>0.3</v>
       </c>
-      <c r="R11" s="91"/>
-      <c r="S11" s="93"/>
+      <c r="R11" s="81"/>
+      <c r="S11" s="83"/>
     </row>
     <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
-      <c r="B12" s="94">
+      <c r="B12" s="84">
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
@@ -2452,13 +2455,13 @@
       <c r="N12" s="45">
         <v>100</v>
       </c>
-      <c r="O12" s="110" t="s">
+      <c r="O12" s="96" t="s">
         <v>193</v>
       </c>
       <c r="P12" s="50">
         <v>4.5999999999999999E-3</v>
       </c>
-      <c r="Q12" s="114">
+      <c r="Q12" s="100">
         <f t="shared" si="2"/>
         <v>0.45999999999999996</v>
       </c>
@@ -2467,63 +2470,63 @@
     </row>
     <row r="13" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
-      <c r="B13" s="94">
+      <c r="B13" s="84">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="88" t="s">
+      <c r="C13" s="78" t="s">
         <v>7</v>
       </c>
-      <c r="D13" s="89" t="s">
+      <c r="D13" s="79" t="s">
         <v>23</v>
       </c>
-      <c r="E13" s="91" t="s">
+      <c r="E13" s="81" t="s">
         <v>55</v>
       </c>
-      <c r="F13" s="91" t="s">
+      <c r="F13" s="81" t="s">
         <v>82</v>
       </c>
-      <c r="G13" s="109" t="s">
+      <c r="G13" s="95" t="s">
         <v>103</v>
       </c>
-      <c r="H13" s="90" t="s">
+      <c r="H13" s="80" t="s">
         <v>125</v>
       </c>
-      <c r="I13" s="91" t="s">
+      <c r="I13" s="81" t="s">
         <v>194</v>
       </c>
-      <c r="J13" s="91" t="s">
+      <c r="J13" s="81" t="s">
         <v>195</v>
       </c>
-      <c r="K13" s="90" t="s">
+      <c r="K13" s="80" t="s">
         <v>164</v>
       </c>
-      <c r="L13" s="91">
+      <c r="L13" s="81">
         <v>1</v>
       </c>
-      <c r="M13" s="90">
+      <c r="M13" s="80">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N13" s="91">
+      <c r="N13" s="81">
         <v>20</v>
       </c>
-      <c r="O13" s="111" t="s">
+      <c r="O13" s="97" t="s">
         <v>193</v>
       </c>
-      <c r="P13" s="92">
+      <c r="P13" s="82">
         <v>2.3400000000000001E-2</v>
       </c>
-      <c r="Q13" s="115">
+      <c r="Q13" s="101">
         <f t="shared" si="2"/>
         <v>0.46800000000000003</v>
       </c>
-      <c r="R13" s="91"/>
-      <c r="S13" s="92"/>
+      <c r="R13" s="81"/>
+      <c r="S13" s="82"/>
     </row>
     <row r="14" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
-      <c r="B14" s="94">
+      <c r="B14" s="84">
         <f>ROW(B14) - ROW($B$9)</f>
         <v>5</v>
       </c>
@@ -2564,13 +2567,13 @@
       <c r="N14" s="45">
         <v>50</v>
       </c>
-      <c r="O14" s="110" t="s">
+      <c r="O14" s="96" t="s">
         <v>193</v>
       </c>
       <c r="P14" s="50">
         <v>1.5599999999999999E-2</v>
       </c>
-      <c r="Q14" s="114">
+      <c r="Q14" s="100">
         <f t="shared" si="2"/>
         <v>0.77999999999999992</v>
       </c>
@@ -2579,66 +2582,66 @@
     </row>
     <row r="15" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
-      <c r="B15" s="94">
+      <c r="B15" s="84">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="88" t="s">
+      <c r="C15" s="78" t="s">
         <v>7</v>
       </c>
-      <c r="D15" s="89" t="s">
+      <c r="D15" s="79" t="s">
         <v>25</v>
       </c>
-      <c r="E15" s="91" t="s">
+      <c r="E15" s="81" t="s">
         <v>57</v>
       </c>
-      <c r="F15" s="91" t="s">
+      <c r="F15" s="81" t="s">
         <v>81</v>
       </c>
-      <c r="G15" s="91" t="s">
-        <v>184</v>
-      </c>
-      <c r="H15" s="90" t="s">
-        <v>184</v>
-      </c>
-      <c r="I15" s="91" t="s">
-        <v>184</v>
-      </c>
-      <c r="J15" s="91" t="s">
-        <v>184</v>
-      </c>
-      <c r="K15" s="90" t="s">
-        <v>184</v>
-      </c>
-      <c r="L15" s="91">
+      <c r="G15" s="81" t="s">
+        <v>184</v>
+      </c>
+      <c r="H15" s="80" t="s">
+        <v>184</v>
+      </c>
+      <c r="I15" s="81" t="s">
+        <v>184</v>
+      </c>
+      <c r="J15" s="81" t="s">
+        <v>184</v>
+      </c>
+      <c r="K15" s="80" t="s">
+        <v>184</v>
+      </c>
+      <c r="L15" s="81">
         <v>2</v>
       </c>
-      <c r="M15" s="90">
+      <c r="M15" s="80">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N15" s="91" t="s">
-        <v>184</v>
-      </c>
-      <c r="O15" s="90" t="s">
-        <v>184</v>
-      </c>
-      <c r="P15" s="91" t="s">
-        <v>184</v>
-      </c>
-      <c r="Q15" s="115" t="s">
-        <v>184</v>
-      </c>
-      <c r="R15" s="91" t="s">
-        <v>184</v>
-      </c>
-      <c r="S15" s="91" t="s">
+      <c r="N15" s="81" t="s">
+        <v>184</v>
+      </c>
+      <c r="O15" s="80" t="s">
+        <v>184</v>
+      </c>
+      <c r="P15" s="81" t="s">
+        <v>184</v>
+      </c>
+      <c r="Q15" s="101" t="s">
+        <v>184</v>
+      </c>
+      <c r="R15" s="81" t="s">
+        <v>184</v>
+      </c>
+      <c r="S15" s="81" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="16" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
-      <c r="B16" s="94">
+      <c r="B16" s="84">
         <f>ROW(B16) - ROW($B$9)</f>
         <v>7</v>
       </c>
@@ -2679,13 +2682,13 @@
       <c r="N16" s="45">
         <v>100</v>
       </c>
-      <c r="O16" s="110" t="s">
+      <c r="O16" s="96" t="s">
         <v>193</v>
       </c>
       <c r="P16" s="50">
         <v>2E-3</v>
       </c>
-      <c r="Q16" s="114">
+      <c r="Q16" s="100">
         <f t="shared" si="2"/>
         <v>0.2</v>
       </c>
@@ -2694,63 +2697,63 @@
     </row>
     <row r="17" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
-      <c r="B17" s="94">
+      <c r="B17" s="84">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="88" t="s">
+      <c r="C17" s="78" t="s">
         <v>7</v>
       </c>
-      <c r="D17" s="89" t="s">
+      <c r="D17" s="79" t="s">
         <v>27</v>
       </c>
-      <c r="E17" s="91" t="s">
+      <c r="E17" s="81" t="s">
         <v>59</v>
       </c>
-      <c r="F17" s="91" t="s">
+      <c r="F17" s="81" t="s">
         <v>81</v>
       </c>
-      <c r="G17" s="91" t="s">
+      <c r="G17" s="81" t="s">
         <v>106</v>
       </c>
-      <c r="H17" s="90" t="s">
+      <c r="H17" s="80" t="s">
         <v>126</v>
       </c>
-      <c r="I17" s="91" t="s">
-        <v>184</v>
-      </c>
-      <c r="J17" s="91" t="s">
+      <c r="I17" s="81" t="s">
+        <v>184</v>
+      </c>
+      <c r="J17" s="81" t="s">
         <v>146</v>
       </c>
-      <c r="K17" s="90" t="s">
+      <c r="K17" s="80" t="s">
         <v>166</v>
       </c>
-      <c r="L17" s="91">
+      <c r="L17" s="81">
         <v>1</v>
       </c>
-      <c r="M17" s="90">
+      <c r="M17" s="80">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N17" s="91">
+      <c r="N17" s="81">
         <v>50</v>
       </c>
-      <c r="O17" s="111" t="s">
+      <c r="O17" s="97" t="s">
         <v>193</v>
       </c>
-      <c r="P17" s="92">
+      <c r="P17" s="82">
         <v>1.3899999999999999E-2</v>
       </c>
-      <c r="Q17" s="115">
+      <c r="Q17" s="101">
         <f t="shared" si="2"/>
         <v>0.69499999999999995</v>
       </c>
-      <c r="R17" s="91"/>
-      <c r="S17" s="92"/>
+      <c r="R17" s="81"/>
+      <c r="S17" s="82"/>
     </row>
     <row r="18" spans="1:19" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
-      <c r="B18" s="94">
+      <c r="B18" s="84">
         <f>ROW(B18) - ROW($B$9)</f>
         <v>9</v>
       </c>
@@ -2791,13 +2794,13 @@
       <c r="N18" s="45">
         <v>40</v>
       </c>
-      <c r="O18" s="110" t="s">
+      <c r="O18" s="96" t="s">
         <v>193</v>
       </c>
       <c r="P18" s="50">
         <v>2.75E-2</v>
       </c>
-      <c r="Q18" s="114">
+      <c r="Q18" s="100">
         <f>P18*N18</f>
         <v>1.1000000000000001</v>
       </c>
@@ -2806,63 +2809,63 @@
     </row>
     <row r="19" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
-      <c r="B19" s="94">
+      <c r="B19" s="84">
         <f>ROW(B19) - ROW($B$9)</f>
         <v>10</v>
       </c>
-      <c r="C19" s="88" t="s">
+      <c r="C19" s="78" t="s">
         <v>188</v>
       </c>
-      <c r="D19" s="89" t="s">
+      <c r="D19" s="79" t="s">
         <v>28</v>
       </c>
-      <c r="E19" s="91" t="s">
+      <c r="E19" s="81" t="s">
         <v>60</v>
       </c>
-      <c r="F19" s="91" t="s">
+      <c r="F19" s="81" t="s">
         <v>84</v>
       </c>
-      <c r="G19" s="91" t="s">
+      <c r="G19" s="81" t="s">
         <v>107</v>
       </c>
-      <c r="H19" s="90" t="s">
+      <c r="H19" s="80" t="s">
         <v>127</v>
       </c>
-      <c r="I19" s="91" t="s">
-        <v>184</v>
-      </c>
-      <c r="J19" s="91" t="s">
+      <c r="I19" s="81" t="s">
+        <v>184</v>
+      </c>
+      <c r="J19" s="81" t="s">
         <v>147</v>
       </c>
-      <c r="K19" s="90" t="s">
-        <v>184</v>
-      </c>
-      <c r="L19" s="91">
+      <c r="K19" s="80" t="s">
+        <v>184</v>
+      </c>
+      <c r="L19" s="81">
         <v>1</v>
       </c>
-      <c r="M19" s="90">
+      <c r="M19" s="80">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N19" s="91">
+      <c r="N19" s="81">
         <v>15</v>
       </c>
-      <c r="O19" s="111" t="s">
+      <c r="O19" s="97" t="s">
         <v>193</v>
       </c>
-      <c r="P19" s="92">
+      <c r="P19" s="82">
         <v>6.54E-2</v>
       </c>
-      <c r="Q19" s="115">
+      <c r="Q19" s="101">
         <f t="shared" si="2"/>
         <v>0.98099999999999998</v>
       </c>
-      <c r="R19" s="91"/>
-      <c r="S19" s="92"/>
+      <c r="R19" s="81"/>
+      <c r="S19" s="82"/>
     </row>
     <row r="20" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
-      <c r="B20" s="94">
+      <c r="B20" s="84">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
@@ -2903,13 +2906,13 @@
       <c r="N20" s="45">
         <v>15</v>
       </c>
-      <c r="O20" s="110" t="s">
+      <c r="O20" s="96" t="s">
         <v>193</v>
       </c>
       <c r="P20" s="50">
         <v>7.1599999999999997E-2</v>
       </c>
-      <c r="Q20" s="114">
+      <c r="Q20" s="100">
         <f t="shared" si="2"/>
         <v>1.0739999999999998</v>
       </c>
@@ -2918,63 +2921,63 @@
     </row>
     <row r="21" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
-      <c r="B21" s="94">
+      <c r="B21" s="84">
         <f>ROW(B21) - ROW($B$9)</f>
         <v>12</v>
       </c>
-      <c r="C21" s="88" t="s">
+      <c r="C21" s="78" t="s">
         <v>189</v>
       </c>
-      <c r="D21" s="89" t="s">
+      <c r="D21" s="79" t="s">
         <v>30</v>
       </c>
-      <c r="E21" s="91" t="s">
+      <c r="E21" s="81" t="s">
         <v>208</v>
       </c>
-      <c r="F21" s="91" t="s">
+      <c r="F21" s="81" t="s">
         <v>185</v>
       </c>
-      <c r="G21" s="91" t="s">
+      <c r="G21" s="81" t="s">
         <v>209</v>
       </c>
-      <c r="H21" s="90" t="s">
+      <c r="H21" s="80" t="s">
         <v>210</v>
       </c>
-      <c r="I21" s="91" t="s">
-        <v>184</v>
-      </c>
-      <c r="J21" s="91" t="s">
+      <c r="I21" s="81" t="s">
+        <v>184</v>
+      </c>
+      <c r="J21" s="81" t="s">
         <v>209</v>
       </c>
-      <c r="K21" s="90" t="s">
-        <v>184</v>
-      </c>
-      <c r="L21" s="91">
+      <c r="K21" s="80" t="s">
+        <v>184</v>
+      </c>
+      <c r="L21" s="81">
         <v>1</v>
       </c>
-      <c r="M21" s="90">
+      <c r="M21" s="80">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N21" s="91">
+      <c r="N21" s="81">
         <v>12</v>
       </c>
-      <c r="O21" s="111" t="s">
+      <c r="O21" s="97" t="s">
         <v>193</v>
       </c>
-      <c r="P21" s="92">
+      <c r="P21" s="82">
         <v>7.1999999999999995E-2</v>
       </c>
-      <c r="Q21" s="115">
+      <c r="Q21" s="101">
         <f t="shared" si="2"/>
         <v>0.86399999999999988</v>
       </c>
-      <c r="R21" s="91"/>
-      <c r="S21" s="92"/>
+      <c r="R21" s="81"/>
+      <c r="S21" s="82"/>
     </row>
     <row r="22" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
-      <c r="B22" s="94">
+      <c r="B22" s="84">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
@@ -3015,13 +3018,13 @@
       <c r="N22" s="45">
         <v>15</v>
       </c>
-      <c r="O22" s="110" t="s">
+      <c r="O22" s="96" t="s">
         <v>193</v>
       </c>
       <c r="P22" s="50">
         <v>0.2276</v>
       </c>
-      <c r="Q22" s="114">
+      <c r="Q22" s="100">
         <f t="shared" si="2"/>
         <v>3.4140000000000001</v>
       </c>
@@ -3030,63 +3033,63 @@
     </row>
     <row r="23" spans="1:19" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
-      <c r="B23" s="94">
+      <c r="B23" s="84">
         <f>ROW(B23) - ROW($B$9)</f>
         <v>14</v>
       </c>
-      <c r="C23" s="88" t="s">
+      <c r="C23" s="78" t="s">
         <v>9</v>
       </c>
-      <c r="D23" s="89" t="s">
+      <c r="D23" s="79" t="s">
         <v>32</v>
       </c>
-      <c r="E23" s="91" t="s">
+      <c r="E23" s="81" t="s">
         <v>211</v>
       </c>
-      <c r="F23" s="91" t="s">
+      <c r="F23" s="81" t="s">
         <v>185</v>
       </c>
-      <c r="G23" s="91" t="s">
+      <c r="G23" s="81" t="s">
         <v>212</v>
       </c>
-      <c r="H23" s="90" t="s">
+      <c r="H23" s="80" t="s">
         <v>213</v>
       </c>
-      <c r="I23" s="91" t="s">
-        <v>184</v>
-      </c>
-      <c r="J23" s="91" t="s">
+      <c r="I23" s="81" t="s">
+        <v>184</v>
+      </c>
+      <c r="J23" s="81" t="s">
         <v>214</v>
       </c>
-      <c r="K23" s="90" t="s">
-        <v>184</v>
-      </c>
-      <c r="L23" s="91">
+      <c r="K23" s="80" t="s">
+        <v>184</v>
+      </c>
+      <c r="L23" s="81">
         <v>1</v>
       </c>
-      <c r="M23" s="90">
+      <c r="M23" s="80">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N23" s="91">
+      <c r="N23" s="81">
         <v>15</v>
       </c>
-      <c r="O23" s="111" t="s">
+      <c r="O23" s="97" t="s">
         <v>193</v>
       </c>
-      <c r="P23" s="92">
+      <c r="P23" s="82">
         <v>6.5600000000000006E-2</v>
       </c>
-      <c r="Q23" s="115">
+      <c r="Q23" s="101">
         <f t="shared" si="2"/>
         <v>0.9840000000000001</v>
       </c>
-      <c r="R23" s="91"/>
-      <c r="S23" s="92"/>
+      <c r="R23" s="81"/>
+      <c r="S23" s="82"/>
     </row>
     <row r="24" spans="1:19" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
-      <c r="B24" s="94">
+      <c r="B24" s="84">
         <f>ROW(B24) - ROW($B$9)</f>
         <v>15</v>
       </c>
@@ -3127,13 +3130,13 @@
       <c r="N24" s="45">
         <v>120</v>
       </c>
-      <c r="O24" s="110" t="s">
+      <c r="O24" s="96" t="s">
         <v>193</v>
       </c>
       <c r="P24" s="50">
         <v>4.6100000000000002E-2</v>
       </c>
-      <c r="Q24" s="114">
+      <c r="Q24" s="100">
         <f>P24*N24</f>
         <v>5.532</v>
       </c>
@@ -3142,63 +3145,63 @@
     </row>
     <row r="25" spans="1:19" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
-      <c r="B25" s="94">
+      <c r="B25" s="84">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C25" s="88" t="s">
+      <c r="C25" s="78" t="s">
         <v>10</v>
       </c>
-      <c r="D25" s="89" t="s">
+      <c r="D25" s="79" t="s">
         <v>33</v>
       </c>
-      <c r="E25" s="91" t="s">
+      <c r="E25" s="81" t="s">
         <v>63</v>
       </c>
-      <c r="F25" s="91" t="s">
+      <c r="F25" s="81" t="s">
         <v>185</v>
       </c>
-      <c r="G25" s="91" t="s">
+      <c r="G25" s="81" t="s">
         <v>86</v>
       </c>
-      <c r="H25" s="90" t="s">
+      <c r="H25" s="80" t="s">
         <v>131</v>
       </c>
-      <c r="I25" s="91" t="s">
-        <v>184</v>
-      </c>
-      <c r="J25" s="91" t="s">
+      <c r="I25" s="81" t="s">
+        <v>184</v>
+      </c>
+      <c r="J25" s="81" t="s">
         <v>150</v>
       </c>
-      <c r="K25" s="90" t="s">
-        <v>184</v>
-      </c>
-      <c r="L25" s="91">
+      <c r="K25" s="80" t="s">
+        <v>184</v>
+      </c>
+      <c r="L25" s="81">
         <v>10</v>
       </c>
-      <c r="M25" s="90">
+      <c r="M25" s="80">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="N25" s="91">
+      <c r="N25" s="81">
         <v>105</v>
       </c>
-      <c r="O25" s="111" t="s">
+      <c r="O25" s="97" t="s">
         <v>193</v>
       </c>
-      <c r="P25" s="92">
+      <c r="P25" s="82">
         <v>0.25779999999999997</v>
       </c>
-      <c r="Q25" s="115">
+      <c r="Q25" s="101">
         <f t="shared" si="2"/>
         <v>27.068999999999996</v>
       </c>
-      <c r="R25" s="91"/>
-      <c r="S25" s="92"/>
+      <c r="R25" s="81"/>
+      <c r="S25" s="82"/>
     </row>
     <row r="26" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
-      <c r="B26" s="94">
+      <c r="B26" s="84">
         <f>ROW(B26) - ROW($B$9)</f>
         <v>17</v>
       </c>
@@ -3239,13 +3242,13 @@
       <c r="N26" s="45">
         <v>110</v>
       </c>
-      <c r="O26" s="110" t="s">
+      <c r="O26" s="96" t="s">
         <v>193</v>
       </c>
       <c r="P26" s="50">
         <v>6.7900000000000002E-2</v>
       </c>
-      <c r="Q26" s="114">
+      <c r="Q26" s="100">
         <f t="shared" si="2"/>
         <v>7.4690000000000003</v>
       </c>
@@ -3254,62 +3257,62 @@
     </row>
     <row r="27" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
-      <c r="B27" s="94">
+      <c r="B27" s="84">
         <f>ROW(B27) - ROW($B$9)</f>
         <v>18</v>
       </c>
-      <c r="C27" s="88" t="s">
+      <c r="C27" s="78" t="s">
         <v>192</v>
       </c>
-      <c r="D27" s="89" t="s">
+      <c r="D27" s="79" t="s">
         <v>35</v>
       </c>
-      <c r="E27" s="91" t="s">
+      <c r="E27" s="81" t="s">
         <v>65</v>
       </c>
-      <c r="F27" s="91" t="s">
+      <c r="F27" s="81" t="s">
         <v>185</v>
       </c>
-      <c r="G27" s="91" t="s">
+      <c r="G27" s="81" t="s">
         <v>88</v>
       </c>
-      <c r="H27" s="90" t="s">
-        <v>184</v>
-      </c>
-      <c r="I27" s="91" t="s">
-        <v>184</v>
-      </c>
-      <c r="J27" s="91" t="s">
-        <v>184</v>
-      </c>
-      <c r="K27" s="90" t="s">
-        <v>184</v>
-      </c>
-      <c r="L27" s="91">
+      <c r="H27" s="80" t="s">
+        <v>184</v>
+      </c>
+      <c r="I27" s="81" t="s">
+        <v>184</v>
+      </c>
+      <c r="J27" s="81" t="s">
+        <v>184</v>
+      </c>
+      <c r="K27" s="80" t="s">
+        <v>184</v>
+      </c>
+      <c r="L27" s="81">
         <v>4</v>
       </c>
-      <c r="M27" s="90">
+      <c r="M27" s="80">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="N27" s="91" t="s">
-        <v>184</v>
-      </c>
-      <c r="O27" s="111" t="s">
-        <v>184</v>
-      </c>
-      <c r="P27" s="92" t="s">
-        <v>184</v>
-      </c>
-      <c r="Q27" s="115" t="s">
-        <v>184</v>
-      </c>
-      <c r="R27" s="91"/>
-      <c r="S27" s="92"/>
+      <c r="N27" s="81" t="s">
+        <v>184</v>
+      </c>
+      <c r="O27" s="97" t="s">
+        <v>184</v>
+      </c>
+      <c r="P27" s="82" t="s">
+        <v>184</v>
+      </c>
+      <c r="Q27" s="101" t="s">
+        <v>184</v>
+      </c>
+      <c r="R27" s="81"/>
+      <c r="S27" s="82"/>
     </row>
     <row r="28" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
-      <c r="B28" s="94">
+      <c r="B28" s="84">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
@@ -3350,13 +3353,13 @@
       <c r="N28" s="45">
         <v>15</v>
       </c>
-      <c r="O28" s="110" t="s">
+      <c r="O28" s="96" t="s">
         <v>193</v>
       </c>
       <c r="P28" s="50">
         <v>6.7400000000000002E-2</v>
       </c>
-      <c r="Q28" s="114">
+      <c r="Q28" s="100">
         <f t="shared" si="2"/>
         <v>1.0110000000000001</v>
       </c>
@@ -3365,63 +3368,63 @@
     </row>
     <row r="29" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
-      <c r="B29" s="94">
+      <c r="B29" s="84">
         <f>ROW(B29) - ROW($B$9)</f>
         <v>20</v>
       </c>
-      <c r="C29" s="88" t="s">
+      <c r="C29" s="78" t="s">
         <v>191</v>
       </c>
-      <c r="D29" s="89" t="s">
+      <c r="D29" s="79" t="s">
         <v>37</v>
       </c>
-      <c r="E29" s="91" t="s">
+      <c r="E29" s="81" t="s">
         <v>67</v>
       </c>
-      <c r="F29" s="91" t="s">
+      <c r="F29" s="81" t="s">
         <v>89</v>
       </c>
-      <c r="G29" s="91" t="s">
+      <c r="G29" s="81" t="s">
         <v>112</v>
       </c>
-      <c r="H29" s="90" t="s">
+      <c r="H29" s="80" t="s">
         <v>134</v>
       </c>
-      <c r="I29" s="91" t="s">
-        <v>184</v>
-      </c>
-      <c r="J29" s="91" t="s">
+      <c r="I29" s="81" t="s">
+        <v>184</v>
+      </c>
+      <c r="J29" s="81" t="s">
         <v>153</v>
       </c>
-      <c r="K29" s="90" t="s">
-        <v>184</v>
-      </c>
-      <c r="L29" s="91">
+      <c r="K29" s="80" t="s">
+        <v>184</v>
+      </c>
+      <c r="L29" s="81">
         <v>1</v>
       </c>
-      <c r="M29" s="90">
+      <c r="M29" s="80">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N29" s="91">
+      <c r="N29" s="81">
         <v>50</v>
       </c>
-      <c r="O29" s="111" t="s">
+      <c r="O29" s="97" t="s">
         <v>193</v>
       </c>
-      <c r="P29" s="92">
+      <c r="P29" s="82">
         <v>1.47E-2</v>
       </c>
-      <c r="Q29" s="115">
+      <c r="Q29" s="101">
         <f t="shared" si="2"/>
         <v>0.73499999999999999</v>
       </c>
-      <c r="R29" s="91"/>
-      <c r="S29" s="92"/>
+      <c r="R29" s="81"/>
+      <c r="S29" s="82"/>
     </row>
     <row r="30" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
-      <c r="B30" s="105">
+      <c r="B30" s="91">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
@@ -3462,13 +3465,13 @@
       <c r="N30" s="71">
         <v>100</v>
       </c>
-      <c r="O30" s="112" t="s">
+      <c r="O30" s="98" t="s">
         <v>193</v>
       </c>
       <c r="P30" s="72">
         <v>1E-3</v>
       </c>
-      <c r="Q30" s="116">
+      <c r="Q30" s="102">
         <f t="shared" si="2"/>
         <v>0.1</v>
       </c>
@@ -3477,63 +3480,63 @@
     </row>
     <row r="31" spans="1:19" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
-      <c r="B31" s="94">
+      <c r="B31" s="84">
         <f>ROW(B31) - ROW($B$9)</f>
         <v>22</v>
       </c>
-      <c r="C31" s="88" t="s">
+      <c r="C31" s="78" t="s">
         <v>12</v>
       </c>
-      <c r="D31" s="91" t="s">
+      <c r="D31" s="81" t="s">
         <v>39</v>
       </c>
-      <c r="E31" s="91" t="s">
+      <c r="E31" s="81" t="s">
         <v>232</v>
       </c>
-      <c r="F31" s="91" t="s">
+      <c r="F31" s="81" t="s">
         <v>233</v>
       </c>
-      <c r="G31" s="91" t="s">
+      <c r="G31" s="81" t="s">
         <v>234</v>
       </c>
-      <c r="H31" s="90" t="s">
+      <c r="H31" s="80" t="s">
         <v>235</v>
       </c>
-      <c r="I31" s="91" t="s">
-        <v>184</v>
-      </c>
-      <c r="J31" s="91" t="s">
+      <c r="I31" s="81" t="s">
+        <v>184</v>
+      </c>
+      <c r="J31" s="81" t="s">
         <v>236</v>
       </c>
-      <c r="K31" s="90" t="s">
+      <c r="K31" s="80" t="s">
         <v>168</v>
       </c>
-      <c r="L31" s="91">
+      <c r="L31" s="81">
         <v>3</v>
       </c>
-      <c r="M31" s="90">
+      <c r="M31" s="80">
         <f t="shared" si="1"/>
         <v>30</v>
       </c>
-      <c r="N31" s="91">
+      <c r="N31" s="81">
         <v>100</v>
       </c>
-      <c r="O31" s="111" t="s">
+      <c r="O31" s="97" t="s">
         <v>193</v>
       </c>
-      <c r="P31" s="92">
+      <c r="P31" s="82">
         <v>6.8999999999999999E-3</v>
       </c>
-      <c r="Q31" s="115">
+      <c r="Q31" s="101">
         <f t="shared" si="2"/>
         <v>0.69</v>
       </c>
-      <c r="R31" s="91"/>
-      <c r="S31" s="92"/>
+      <c r="R31" s="81"/>
+      <c r="S31" s="82"/>
     </row>
     <row r="32" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
-      <c r="B32" s="94">
+      <c r="B32" s="84">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
@@ -3574,13 +3577,13 @@
       <c r="N32" s="45">
         <v>50</v>
       </c>
-      <c r="O32" s="110" t="s">
+      <c r="O32" s="96" t="s">
         <v>193</v>
       </c>
       <c r="P32" s="50">
         <v>7.7999999999999996E-3</v>
       </c>
-      <c r="Q32" s="114">
+      <c r="Q32" s="100">
         <f t="shared" si="2"/>
         <v>0.38999999999999996</v>
       </c>
@@ -3589,63 +3592,63 @@
     </row>
     <row r="33" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
-      <c r="B33" s="94">
+      <c r="B33" s="84">
         <f>ROW(B33) - ROW($B$9)</f>
         <v>24</v>
       </c>
-      <c r="C33" s="88" t="s">
+      <c r="C33" s="78" t="s">
         <v>13</v>
       </c>
-      <c r="D33" s="89" t="s">
+      <c r="D33" s="79" t="s">
         <v>41</v>
       </c>
-      <c r="E33" s="91" t="s">
+      <c r="E33" s="81" t="s">
         <v>69</v>
       </c>
-      <c r="F33" s="91" t="s">
+      <c r="F33" s="81" t="s">
         <v>91</v>
       </c>
-      <c r="G33" s="109" t="s">
+      <c r="G33" s="95" t="s">
         <v>114</v>
       </c>
-      <c r="H33" s="90" t="s">
+      <c r="H33" s="80" t="s">
         <v>135</v>
       </c>
-      <c r="I33" s="91" t="s">
+      <c r="I33" s="81" t="s">
         <v>197</v>
       </c>
-      <c r="J33" s="91" t="s">
+      <c r="J33" s="81" t="s">
         <v>196</v>
       </c>
-      <c r="K33" s="90" t="s">
+      <c r="K33" s="80" t="s">
         <v>170</v>
       </c>
-      <c r="L33" s="91">
+      <c r="L33" s="81">
         <v>2</v>
       </c>
-      <c r="M33" s="90">
+      <c r="M33" s="80">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N33" s="91">
+      <c r="N33" s="81">
         <v>100</v>
       </c>
-      <c r="O33" s="111" t="s">
+      <c r="O33" s="97" t="s">
         <v>193</v>
       </c>
-      <c r="P33" s="92">
+      <c r="P33" s="82">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="Q33" s="115">
+      <c r="Q33" s="101">
         <f t="shared" si="2"/>
         <v>0.05</v>
       </c>
-      <c r="R33" s="91"/>
-      <c r="S33" s="92"/>
+      <c r="R33" s="81"/>
+      <c r="S33" s="82"/>
     </row>
     <row r="34" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
-      <c r="B34" s="94">
+      <c r="B34" s="84">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
@@ -3686,13 +3689,13 @@
       <c r="N34" s="45">
         <v>100</v>
       </c>
-      <c r="O34" s="110" t="s">
+      <c r="O34" s="96" t="s">
         <v>193</v>
       </c>
       <c r="P34" s="50">
         <v>1.4E-3</v>
       </c>
-      <c r="Q34" s="114">
+      <c r="Q34" s="100">
         <f t="shared" si="2"/>
         <v>0.13999999999999999</v>
       </c>
@@ -3701,63 +3704,63 @@
     </row>
     <row r="35" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
-      <c r="B35" s="94">
+      <c r="B35" s="84">
         <f>ROW(B35) - ROW($B$9)</f>
         <v>26</v>
       </c>
-      <c r="C35" s="88" t="s">
+      <c r="C35" s="78" t="s">
         <v>13</v>
       </c>
-      <c r="D35" s="89" t="s">
+      <c r="D35" s="79" t="s">
         <v>43</v>
       </c>
-      <c r="E35" s="91" t="s">
+      <c r="E35" s="81" t="s">
         <v>71</v>
       </c>
-      <c r="F35" s="91" t="s">
+      <c r="F35" s="81" t="s">
         <v>91</v>
       </c>
-      <c r="G35" s="91" t="s">
+      <c r="G35" s="81" t="s">
         <v>116</v>
       </c>
-      <c r="H35" s="90" t="s">
+      <c r="H35" s="80" t="s">
         <v>126</v>
       </c>
-      <c r="I35" s="91" t="s">
-        <v>184</v>
-      </c>
-      <c r="J35" s="91" t="s">
+      <c r="I35" s="81" t="s">
+        <v>184</v>
+      </c>
+      <c r="J35" s="81" t="s">
         <v>198</v>
       </c>
-      <c r="K35" s="90" t="s">
+      <c r="K35" s="80" t="s">
         <v>172</v>
       </c>
-      <c r="L35" s="91">
+      <c r="L35" s="81">
         <v>1</v>
       </c>
-      <c r="M35" s="90">
+      <c r="M35" s="80">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N35" s="91">
+      <c r="N35" s="81">
         <v>100</v>
       </c>
-      <c r="O35" s="111" t="s">
+      <c r="O35" s="97" t="s">
         <v>193</v>
       </c>
-      <c r="P35" s="92">
+      <c r="P35" s="82">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="Q35" s="115">
+      <c r="Q35" s="101">
         <f t="shared" si="2"/>
         <v>0.05</v>
       </c>
-      <c r="R35" s="91"/>
-      <c r="S35" s="92"/>
+      <c r="R35" s="81"/>
+      <c r="S35" s="82"/>
     </row>
     <row r="36" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
-      <c r="B36" s="94">
+      <c r="B36" s="84">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
@@ -3798,13 +3801,13 @@
       <c r="N36" s="45">
         <v>200</v>
       </c>
-      <c r="O36" s="110" t="s">
+      <c r="O36" s="96" t="s">
         <v>193</v>
       </c>
       <c r="P36" s="50">
         <v>6.9999999999999999E-4</v>
       </c>
-      <c r="Q36" s="114">
+      <c r="Q36" s="100">
         <f t="shared" si="2"/>
         <v>0.13999999999999999</v>
       </c>
@@ -3813,63 +3816,63 @@
     </row>
     <row r="37" spans="1:19" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
-      <c r="B37" s="94">
+      <c r="B37" s="84">
         <f>ROW(B37) - ROW($B$9)</f>
         <v>28</v>
       </c>
-      <c r="C37" s="88" t="s">
+      <c r="C37" s="78" t="s">
         <v>14</v>
       </c>
-      <c r="D37" s="89" t="s">
+      <c r="D37" s="79" t="s">
         <v>45</v>
       </c>
-      <c r="E37" s="91" t="s">
+      <c r="E37" s="81" t="s">
         <v>73</v>
       </c>
-      <c r="F37" s="91" t="s">
+      <c r="F37" s="81" t="s">
         <v>185</v>
       </c>
-      <c r="G37" s="91" t="s">
+      <c r="G37" s="81" t="s">
         <v>93</v>
       </c>
-      <c r="H37" s="90" t="s">
+      <c r="H37" s="80" t="s">
         <v>136</v>
       </c>
-      <c r="I37" s="91" t="s">
-        <v>184</v>
-      </c>
-      <c r="J37" s="91" t="s">
+      <c r="I37" s="81" t="s">
+        <v>184</v>
+      </c>
+      <c r="J37" s="81" t="s">
         <v>156</v>
       </c>
-      <c r="K37" s="90" t="s">
-        <v>184</v>
-      </c>
-      <c r="L37" s="91">
+      <c r="K37" s="80" t="s">
+        <v>184</v>
+      </c>
+      <c r="L37" s="81">
         <v>1</v>
       </c>
-      <c r="M37" s="90">
+      <c r="M37" s="80">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N37" s="91">
+      <c r="N37" s="81">
         <v>20</v>
       </c>
-      <c r="O37" s="111" t="s">
+      <c r="O37" s="97" t="s">
         <v>193</v>
       </c>
-      <c r="P37" s="92">
+      <c r="P37" s="82">
         <v>1.7999999999999999E-2</v>
       </c>
-      <c r="Q37" s="115">
+      <c r="Q37" s="101">
         <f t="shared" si="2"/>
         <v>0.36</v>
       </c>
-      <c r="R37" s="91"/>
-      <c r="S37" s="92"/>
+      <c r="R37" s="81"/>
+      <c r="S37" s="82"/>
     </row>
     <row r="38" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
-      <c r="B38" s="94">
+      <c r="B38" s="84">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
@@ -3910,13 +3913,13 @@
       <c r="N38" s="45">
         <v>11</v>
       </c>
-      <c r="O38" s="110" t="s">
+      <c r="O38" s="96" t="s">
         <v>193</v>
       </c>
       <c r="P38" s="50">
         <v>3.3553000000000002</v>
       </c>
-      <c r="Q38" s="114">
+      <c r="Q38" s="100">
         <f t="shared" si="2"/>
         <v>36.908300000000004</v>
       </c>
@@ -3925,63 +3928,63 @@
     </row>
     <row r="39" spans="1:19" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
-      <c r="B39" s="94">
+      <c r="B39" s="84">
         <f>ROW(B39) - ROW($B$9)</f>
         <v>30</v>
       </c>
-      <c r="C39" s="88" t="s">
+      <c r="C39" s="78" t="s">
         <v>16</v>
       </c>
-      <c r="D39" s="89" t="s">
+      <c r="D39" s="79" t="s">
         <v>47</v>
       </c>
-      <c r="E39" s="91" t="s">
+      <c r="E39" s="81" t="s">
         <v>75</v>
       </c>
-      <c r="F39" s="91" t="s">
+      <c r="F39" s="81" t="s">
         <v>95</v>
       </c>
-      <c r="G39" s="91" t="s">
+      <c r="G39" s="81" t="s">
         <v>119</v>
       </c>
-      <c r="H39" s="90" t="s">
+      <c r="H39" s="80" t="s">
         <v>138</v>
       </c>
-      <c r="I39" s="91" t="s">
-        <v>184</v>
-      </c>
-      <c r="J39" s="91" t="s">
+      <c r="I39" s="81" t="s">
+        <v>184</v>
+      </c>
+      <c r="J39" s="81" t="s">
         <v>158</v>
       </c>
-      <c r="K39" s="90" t="s">
-        <v>184</v>
-      </c>
-      <c r="L39" s="91">
+      <c r="K39" s="80" t="s">
+        <v>184</v>
+      </c>
+      <c r="L39" s="81">
         <v>1</v>
       </c>
-      <c r="M39" s="90">
+      <c r="M39" s="80">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N39" s="91">
+      <c r="N39" s="81">
         <v>11</v>
       </c>
-      <c r="O39" s="111" t="s">
+      <c r="O39" s="97" t="s">
         <v>193</v>
       </c>
-      <c r="P39" s="92">
+      <c r="P39" s="82">
         <v>0.70960000000000001</v>
       </c>
-      <c r="Q39" s="115">
+      <c r="Q39" s="101">
         <f t="shared" si="2"/>
         <v>7.8056000000000001</v>
       </c>
-      <c r="R39" s="91"/>
-      <c r="S39" s="92"/>
+      <c r="R39" s="81"/>
+      <c r="S39" s="82"/>
     </row>
     <row r="40" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
-      <c r="B40" s="94">
+      <c r="B40" s="84">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
@@ -4022,13 +4025,13 @@
       <c r="N40" s="45">
         <v>105</v>
       </c>
-      <c r="O40" s="110" t="s">
+      <c r="O40" s="96" t="s">
         <v>193</v>
       </c>
       <c r="P40" s="50">
         <v>0.11749999999999999</v>
       </c>
-      <c r="Q40" s="114">
+      <c r="Q40" s="100">
         <f t="shared" si="2"/>
         <v>12.337499999999999</v>
       </c>
@@ -4037,63 +4040,63 @@
     </row>
     <row r="41" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
-      <c r="B41" s="94">
+      <c r="B41" s="84">
         <f>ROW(B41) - ROW($B$9)</f>
         <v>32</v>
       </c>
-      <c r="C41" s="88" t="s">
+      <c r="C41" s="78" t="s">
         <v>18</v>
       </c>
-      <c r="D41" s="89" t="s">
+      <c r="D41" s="79" t="s">
         <v>49</v>
       </c>
-      <c r="E41" s="91" t="s">
+      <c r="E41" s="81" t="s">
         <v>77</v>
       </c>
-      <c r="F41" s="91" t="s">
+      <c r="F41" s="81" t="s">
         <v>97</v>
       </c>
-      <c r="G41" s="91" t="s">
+      <c r="G41" s="81" t="s">
         <v>121</v>
       </c>
-      <c r="H41" s="90" t="s">
+      <c r="H41" s="80" t="s">
         <v>140</v>
       </c>
-      <c r="I41" s="91" t="s">
-        <v>184</v>
-      </c>
-      <c r="J41" s="91" t="s">
+      <c r="I41" s="81" t="s">
+        <v>184</v>
+      </c>
+      <c r="J41" s="81" t="s">
         <v>160</v>
       </c>
-      <c r="K41" s="90" t="s">
-        <v>184</v>
-      </c>
-      <c r="L41" s="91">
+      <c r="K41" s="80" t="s">
+        <v>184</v>
+      </c>
+      <c r="L41" s="81">
         <v>1</v>
       </c>
-      <c r="M41" s="90">
+      <c r="M41" s="80">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N41" s="91">
+      <c r="N41" s="81">
         <v>15</v>
       </c>
-      <c r="O41" s="111" t="s">
+      <c r="O41" s="97" t="s">
         <v>193</v>
       </c>
-      <c r="P41" s="92">
+      <c r="P41" s="82">
         <v>0.3513</v>
       </c>
-      <c r="Q41" s="115">
+      <c r="Q41" s="101">
         <f t="shared" si="2"/>
         <v>5.2694999999999999</v>
       </c>
-      <c r="R41" s="91"/>
-      <c r="S41" s="92"/>
+      <c r="R41" s="81"/>
+      <c r="S41" s="82"/>
     </row>
     <row r="42" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
-      <c r="B42" s="94">
+      <c r="B42" s="84">
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
@@ -4134,13 +4137,13 @@
       <c r="N42" s="45">
         <v>25</v>
       </c>
-      <c r="O42" s="110" t="s">
+      <c r="O42" s="96" t="s">
         <v>193</v>
       </c>
       <c r="P42" s="50">
         <v>8.1199999999999994E-2</v>
       </c>
-      <c r="Q42" s="114">
+      <c r="Q42" s="100">
         <f t="shared" si="2"/>
         <v>2.0299999999999998</v>
       </c>
@@ -4149,255 +4152,255 @@
     </row>
     <row r="43" spans="1:19" s="75" customFormat="1" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="73"/>
-      <c r="B43" s="94">
+      <c r="B43" s="84">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="C43" s="88" t="s">
+      <c r="C43" s="78" t="s">
+        <v>9</v>
+      </c>
+      <c r="D43" s="79" t="s">
+        <v>184</v>
+      </c>
+      <c r="E43" s="81" t="s">
+        <v>240</v>
+      </c>
+      <c r="F43" s="81" t="s">
+        <v>185</v>
+      </c>
+      <c r="G43" s="81" t="s">
         <v>237</v>
       </c>
-      <c r="D43" s="89" t="s">
-        <v>184</v>
-      </c>
-      <c r="E43" s="91" t="s">
-        <v>241</v>
-      </c>
-      <c r="F43" s="91" t="s">
-        <v>185</v>
-      </c>
-      <c r="G43" s="91" t="s">
+      <c r="H43" s="80" t="s">
+        <v>130</v>
+      </c>
+      <c r="I43" s="81" t="s">
+        <v>184</v>
+      </c>
+      <c r="J43" s="81" t="s">
         <v>238</v>
       </c>
-      <c r="H43" s="90" t="s">
-        <v>130</v>
-      </c>
-      <c r="I43" s="91" t="s">
-        <v>184</v>
-      </c>
-      <c r="J43" s="91" t="s">
-        <v>239</v>
-      </c>
-      <c r="K43" s="90" t="s">
-        <v>184</v>
-      </c>
-      <c r="L43" s="91">
+      <c r="K43" s="80" t="s">
+        <v>184</v>
+      </c>
+      <c r="L43" s="81">
         <v>11</v>
       </c>
-      <c r="M43" s="90">
+      <c r="M43" s="80">
         <f t="shared" si="1"/>
         <v>110</v>
       </c>
-      <c r="N43" s="91">
+      <c r="N43" s="81">
         <v>115</v>
       </c>
-      <c r="O43" s="111" t="s">
+      <c r="O43" s="97" t="s">
         <v>193</v>
       </c>
-      <c r="P43" s="92">
+      <c r="P43" s="82">
         <v>0.1517</v>
       </c>
-      <c r="Q43" s="115">
+      <c r="Q43" s="101">
         <f t="shared" si="2"/>
         <v>17.445499999999999</v>
       </c>
-      <c r="R43" s="91"/>
-      <c r="S43" s="92"/>
+      <c r="R43" s="81"/>
+      <c r="S43" s="82"/>
     </row>
     <row r="44" spans="1:19" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
-      <c r="B44" s="94">
+      <c r="B44" s="84">
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
-      <c r="C44" s="88" t="s">
-        <v>237</v>
-      </c>
-      <c r="D44" s="89" t="s">
-        <v>184</v>
-      </c>
-      <c r="E44" s="91" t="s">
+      <c r="C44" s="78" t="s">
+        <v>9</v>
+      </c>
+      <c r="D44" s="79" t="s">
+        <v>184</v>
+      </c>
+      <c r="E44" s="81" t="s">
+        <v>241</v>
+      </c>
+      <c r="F44" s="81" t="s">
+        <v>185</v>
+      </c>
+      <c r="G44" s="81" t="s">
+        <v>239</v>
+      </c>
+      <c r="H44" s="80" t="s">
         <v>242</v>
       </c>
-      <c r="F44" s="91" t="s">
-        <v>185</v>
-      </c>
-      <c r="G44" s="91" t="s">
-        <v>240</v>
-      </c>
-      <c r="H44" s="90" t="s">
+      <c r="I44" s="81" t="s">
+        <v>184</v>
+      </c>
+      <c r="J44" s="81" t="s">
         <v>243</v>
       </c>
-      <c r="I44" s="91" t="s">
-        <v>184</v>
-      </c>
-      <c r="J44" s="91" t="s">
-        <v>244</v>
-      </c>
-      <c r="K44" s="90" t="s">
-        <v>184</v>
-      </c>
-      <c r="L44" s="91">
+      <c r="K44" s="80" t="s">
+        <v>184</v>
+      </c>
+      <c r="L44" s="81">
         <v>1</v>
       </c>
-      <c r="M44" s="90">
+      <c r="M44" s="80">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N44" s="91">
+      <c r="N44" s="81">
         <v>15</v>
       </c>
-      <c r="O44" s="111" t="s">
+      <c r="O44" s="97" t="s">
         <v>193</v>
       </c>
-      <c r="P44" s="92">
+      <c r="P44" s="82">
         <v>0.34610000000000002</v>
       </c>
-      <c r="Q44" s="115">
+      <c r="Q44" s="101">
         <f t="shared" si="2"/>
         <v>5.1915000000000004</v>
       </c>
-      <c r="R44" s="91"/>
-      <c r="S44" s="92"/>
+      <c r="R44" s="81"/>
+      <c r="S44" s="82"/>
     </row>
     <row r="45" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1"/>
-      <c r="B45" s="94">
+      <c r="B45" s="84">
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="C45" s="88" t="s">
-        <v>237</v>
-      </c>
-      <c r="D45" s="89" t="s">
-        <v>184</v>
-      </c>
-      <c r="E45" s="91" t="s">
+      <c r="C45" s="78" t="s">
+        <v>254</v>
+      </c>
+      <c r="D45" s="79" t="s">
+        <v>184</v>
+      </c>
+      <c r="E45" s="81" t="s">
+        <v>247</v>
+      </c>
+      <c r="F45" s="81" t="s">
+        <v>185</v>
+      </c>
+      <c r="G45" s="81" t="s">
+        <v>244</v>
+      </c>
+      <c r="H45" s="80" t="s">
         <v>248</v>
       </c>
-      <c r="F45" s="91" t="s">
-        <v>185</v>
-      </c>
-      <c r="G45" s="91" t="s">
-        <v>245</v>
-      </c>
-      <c r="H45" s="90" t="s">
-        <v>249</v>
-      </c>
-      <c r="I45" s="91" t="s">
-        <v>184</v>
-      </c>
-      <c r="J45" s="91" t="s">
-        <v>252</v>
-      </c>
-      <c r="K45" s="90" t="s">
-        <v>184</v>
-      </c>
-      <c r="L45" s="91">
+      <c r="I45" s="81" t="s">
+        <v>184</v>
+      </c>
+      <c r="J45" s="81" t="s">
+        <v>251</v>
+      </c>
+      <c r="K45" s="80" t="s">
+        <v>184</v>
+      </c>
+      <c r="L45" s="81">
         <v>1</v>
       </c>
-      <c r="M45" s="90">
+      <c r="M45" s="80">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N45" s="91">
+      <c r="N45" s="81">
         <v>11</v>
       </c>
-      <c r="O45" s="111" t="s">
+      <c r="O45" s="97" t="s">
         <v>193</v>
       </c>
-      <c r="P45" s="92">
+      <c r="P45" s="82">
         <v>0.68320000000000003</v>
       </c>
-      <c r="Q45" s="115">
+      <c r="Q45" s="101">
         <f t="shared" si="2"/>
         <v>7.5152000000000001</v>
       </c>
-      <c r="R45" s="91"/>
-      <c r="S45" s="92"/>
+      <c r="R45" s="81"/>
+      <c r="S45" s="82"/>
     </row>
     <row r="46" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
-        <v>254</v>
-      </c>
-      <c r="B46" s="94">
+        <v>253</v>
+      </c>
+      <c r="B46" s="84">
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
-      <c r="C46" s="106" t="s">
-        <v>237</v>
-      </c>
-      <c r="D46" s="107" t="s">
-        <v>184</v>
-      </c>
-      <c r="E46" s="108" t="s">
-        <v>247</v>
-      </c>
-      <c r="F46" s="108" t="s">
+      <c r="C46" s="92" t="s">
+        <v>255</v>
+      </c>
+      <c r="D46" s="93" t="s">
+        <v>184</v>
+      </c>
+      <c r="E46" s="94" t="s">
+        <v>246</v>
+      </c>
+      <c r="F46" s="94" t="s">
         <v>185</v>
       </c>
-      <c r="G46" s="108" t="s">
-        <v>246</v>
-      </c>
-      <c r="H46" s="118" t="s">
+      <c r="G46" s="94" t="s">
+        <v>245</v>
+      </c>
+      <c r="H46" s="104" t="s">
+        <v>249</v>
+      </c>
+      <c r="I46" s="94" t="s">
+        <v>184</v>
+      </c>
+      <c r="J46" s="94" t="s">
         <v>250</v>
       </c>
-      <c r="I46" s="108" t="s">
-        <v>184</v>
-      </c>
-      <c r="J46" s="108" t="s">
-        <v>251</v>
-      </c>
-      <c r="K46" s="118" t="s">
-        <v>184</v>
-      </c>
-      <c r="L46" s="108">
+      <c r="K46" s="104" t="s">
+        <v>184</v>
+      </c>
+      <c r="L46" s="94">
         <v>1</v>
       </c>
-      <c r="M46" s="118">
+      <c r="M46" s="104">
         <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="N46" s="108">
+      <c r="N46" s="94">
         <v>11</v>
       </c>
-      <c r="O46" s="119" t="s">
+      <c r="O46" s="105" t="s">
         <v>193</v>
       </c>
-      <c r="P46" s="113">
+      <c r="P46" s="99">
         <v>0.96099999999999997</v>
       </c>
-      <c r="Q46" s="120">
+      <c r="Q46" s="106">
         <f t="shared" si="2"/>
         <v>10.571</v>
       </c>
-      <c r="R46" s="108"/>
-      <c r="S46" s="113"/>
+      <c r="R46" s="94"/>
+      <c r="S46" s="99"/>
     </row>
     <row r="47" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="1"/>
-      <c r="B47" s="117"/>
-      <c r="C47" s="95"/>
-      <c r="D47" s="96"/>
-      <c r="E47" s="97"/>
-      <c r="F47" s="98"/>
-      <c r="G47" s="99"/>
-      <c r="H47" s="98"/>
-      <c r="I47" s="99"/>
-      <c r="J47" s="98"/>
-      <c r="K47" s="99"/>
-      <c r="L47" s="99"/>
-      <c r="M47" s="99"/>
-      <c r="N47" s="100" t="s">
+      <c r="B47" s="103"/>
+      <c r="C47" s="85"/>
+      <c r="D47" s="86"/>
+      <c r="E47" s="87"/>
+      <c r="F47" s="88"/>
+      <c r="G47" s="89"/>
+      <c r="H47" s="88"/>
+      <c r="I47" s="89"/>
+      <c r="J47" s="88"/>
+      <c r="K47" s="89"/>
+      <c r="L47" s="89"/>
+      <c r="M47" s="89"/>
+      <c r="N47" s="115" t="s">
         <v>220</v>
       </c>
-      <c r="O47" s="101"/>
-      <c r="P47" s="101"/>
-      <c r="Q47" s="102">
+      <c r="O47" s="116"/>
+      <c r="P47" s="116"/>
+      <c r="Q47" s="90">
         <f>SUM(Q10:Q46)</f>
         <v>161.08609999999999</v>
       </c>
-      <c r="R47" s="103"/>
-      <c r="S47" s="104"/>
+      <c r="R47" s="111"/>
+      <c r="S47" s="112"/>
     </row>
     <row r="48" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A48" s="1"/>
@@ -4413,17 +4416,17 @@
       <c r="K48" s="10"/>
       <c r="L48" s="10"/>
       <c r="M48" s="10"/>
-      <c r="N48" s="85" t="s">
+      <c r="N48" s="117" t="s">
         <v>221</v>
       </c>
-      <c r="O48" s="86"/>
-      <c r="P48" s="86"/>
+      <c r="O48" s="118"/>
+      <c r="P48" s="118"/>
       <c r="Q48" s="67">
         <f>Q47/10</f>
         <v>16.108609999999999</v>
       </c>
-      <c r="R48" s="83"/>
-      <c r="S48" s="84"/>
+      <c r="R48" s="113"/>
+      <c r="S48" s="114"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -4511,15 +4514,15 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="77"/>
-      <c r="L1" s="77"/>
-      <c r="M1" s="77"/>
-      <c r="N1" s="77"/>
-      <c r="O1" s="77"/>
-      <c r="P1" s="77"/>
-      <c r="Q1" s="77"/>
-      <c r="R1" s="77"/>
-      <c r="S1" s="78"/>
+      <c r="K1" s="107"/>
+      <c r="L1" s="107"/>
+      <c r="M1" s="107"/>
+      <c r="N1" s="107"/>
+      <c r="O1" s="107"/>
+      <c r="P1" s="107"/>
+      <c r="Q1" s="107"/>
+      <c r="R1" s="107"/>
+      <c r="S1" s="108"/>
     </row>
     <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -4569,7 +4572,7 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="5"/>
-      <c r="S3" s="79"/>
+      <c r="S3" s="109"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -4594,7 +4597,7 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
-      <c r="S4" s="80"/>
+      <c r="S4" s="110"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -4619,7 +4622,7 @@
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
       <c r="R5" s="6"/>
-      <c r="S5" s="80"/>
+      <c r="S5" s="110"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -4640,7 +4643,7 @@
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
-      <c r="S6" s="80"/>
+      <c r="S6" s="110"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -4661,7 +4664,7 @@
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
-      <c r="S7" s="80"/>
+      <c r="S7" s="110"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -4682,7 +4685,7 @@
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
-      <c r="S8" s="80"/>
+      <c r="S8" s="110"/>
     </row>
     <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -6605,17 +6608,17 @@
       <c r="K43" s="36"/>
       <c r="L43" s="36"/>
       <c r="M43" s="36"/>
-      <c r="N43" s="85" t="s">
+      <c r="N43" s="117" t="s">
         <v>220</v>
       </c>
-      <c r="O43" s="86"/>
-      <c r="P43" s="86"/>
+      <c r="O43" s="118"/>
+      <c r="P43" s="118"/>
       <c r="Q43" s="66">
         <f>SUM(Q10:Q42)</f>
         <v>9771.9939999999988</v>
       </c>
-      <c r="R43" s="81"/>
-      <c r="S43" s="82"/>
+      <c r="R43" s="119"/>
+      <c r="S43" s="120"/>
     </row>
     <row r="44" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
@@ -6631,17 +6634,17 @@
       <c r="K44" s="10"/>
       <c r="L44" s="10"/>
       <c r="M44" s="10"/>
-      <c r="N44" s="85" t="s">
+      <c r="N44" s="117" t="s">
         <v>221</v>
       </c>
-      <c r="O44" s="86"/>
-      <c r="P44" s="86"/>
+      <c r="O44" s="118"/>
+      <c r="P44" s="118"/>
       <c r="Q44" s="67">
         <f>Q43/1000</f>
         <v>9.7719939999999994</v>
       </c>
-      <c r="R44" s="83"/>
-      <c r="S44" s="84"/>
+      <c r="R44" s="113"/>
+      <c r="S44" s="114"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>